<commit_message>
Production release: full framework promotion 2026-03-01
</commit_message>
<xml_diff>
--- a/isms-core-framework/A.5-organisational-controls/isms-a.5.31-legal-statutory-regulatory-contractual-requirements/WKBK/ISMS-IMP-A.5.31.4_Control_Mapping_20260301.xlsx
+++ b/isms-core-framework/A.5-organisational-controls/isms-a.5.31-legal-statutory-regulatory-contractual-requirements/WKBK/ISMS-IMP-A.5.31.4_Control_Mapping_20260301.xlsx
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,35 +91,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FF9900"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="0000B050"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00003366"/>
@@ -143,7 +114,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -179,12 +150,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00003366"/>
         <bgColor rgb="00003366"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -288,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -339,67 +304,58 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6300,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6351,17 +6307,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>REG-ISO27001-8.1-001</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Implement Annex A controls</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Technical</t>
         </is>
@@ -6376,117 +6332,28 @@
           <t>❌ Complete Gap</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>This is a meta-requirement covering all 93 controls. Gap analysis shows 28 controls not yet implemented.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>GAP SUMMARY STATISTICS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>Total Requirements Mapped:</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>Complete Gaps (No Primary Mapping):</t>
-        </is>
-      </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>Partial Gaps (Only Secondary/Supporting):</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>No Gaps (Primary Mapping Exists):</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>High High Priority Gaps:</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>Medium Medium Priority Gaps:</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>Low Low Priority Gaps:</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>NOTE: This is sample data. In production use, formulas would auto-calculate gaps from the mapping matrix.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:F2"/>
-  <mergeCells count="3">
-    <mergeCell ref="A6:F6"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A18:F18"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="C4:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Technical,Organisational,Legal/Regulatory,Operational,Physical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D4:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"❌ Complete Gap,⚠ Partial Gap,✅ No Gap"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6510,326 +6377,326 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>CONTROL MAPPING — SUMMARY DASHBOARD</t>
         </is>
       </c>
-      <c r="B1" s="28" t="n"/>
-      <c r="C1" s="28" t="n"/>
-      <c r="D1" s="28" t="n"/>
-      <c r="E1" s="28" t="n"/>
-      <c r="F1" s="28" t="n"/>
-      <c r="G1" s="28" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 — Control A.5.31: Legal, Statutory, Regulatory and Contractual Requirements | Control Mapping</t>
         </is>
       </c>
-      <c r="B2" s="28" t="n"/>
-      <c r="C2" s="28" t="n"/>
-      <c r="D2" s="28" t="n"/>
-      <c r="E2" s="28" t="n"/>
-      <c r="F2" s="28" t="n"/>
-      <c r="G2" s="28" t="n"/>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="21" t="n"/>
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="21" t="n"/>
+      <c r="G2" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>TABLE 1: ASSESSMENT AREA COMPLIANCE OVERVIEW</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n"/>
-      <c r="C4" s="28" t="n"/>
-      <c r="D4" s="28" t="n"/>
-      <c r="E4" s="28" t="n"/>
-      <c r="F4" s="28" t="n"/>
-      <c r="G4" s="28" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="21" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Assessment Area</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Total Items</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Non-Compliant</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Compliance %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Control Mapping Coverage</t>
         </is>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="26">
         <f>COUNTA('Control Mapping Matrix'!A3:A1000)</f>
         <v/>
       </c>
-      <c r="C6" s="33">
-        <f>B6-COUNTA('Gap Summary'!A3:A1000)</f>
+      <c r="C6" s="26">
+        <f>B6-COUNTA('Gap Summary'!A4:A1000)</f>
         <v/>
       </c>
-      <c r="D6" s="33" t="n">
+      <c r="D6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="33">
-        <f>COUNTA('Gap Summary'!A3:A1000)</f>
+      <c r="E6" s="26">
+        <f>COUNTA('Gap Summary'!A4:A1000)</f>
         <v/>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="27">
         <f>IFERROR(IF((B6-F6)=0,0,C6/(B6-F6)),"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="36">
+      <c r="B7" s="29">
         <f>SUM(B6:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="29">
         <f>SUM(C6:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="29">
         <f>SUM(D6:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="36">
+      <c r="E7" s="29">
         <f>SUM(E6:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="36">
+      <c r="F7" s="29">
         <f>SUM(F6:F6)</f>
         <v/>
       </c>
-      <c r="G7" s="37">
+      <c r="G7" s="30">
         <f>IFERROR(IF((B7-F7)=0,0,C7/(B7-F7)),"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>TABLE 2: KEY METRICS</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n"/>
-      <c r="C9" s="28" t="n"/>
-      <c r="D9" s="28" t="n"/>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C10" s="31" t="n"/>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="31" t="n"/>
-      <c r="G10" s="31" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Total requirements in scope</t>
         </is>
       </c>
-      <c r="B11" s="33">
+      <c r="B11" s="26">
         <f>COUNTA('Control Mapping Matrix'!A3:A1000)</f>
         <v/>
       </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="28" t="n"/>
-      <c r="G11" s="28" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Requirements with Primary control mapped</t>
         </is>
       </c>
-      <c r="B12" s="33">
-        <f>B6-COUNTA('Gap Summary'!A3:A1000)</f>
+      <c r="B12" s="26">
+        <f>B6-COUNTA('Gap Summary'!A4:A1000)</f>
         <v/>
       </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
-      <c r="G12" s="28" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Requirements in gap analysis</t>
         </is>
       </c>
-      <c r="B13" s="33">
-        <f>COUNTA('Gap Summary'!A3:A1000)</f>
+      <c r="B13" s="26">
+        <f>COUNTA('Gap Summary'!A4:A1000)</f>
         <v/>
       </c>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="28" t="n"/>
-      <c r="G13" s="28" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Total ISO 27001 controls referenced</t>
         </is>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="26">
         <f>COUNTA('ISO27001 Controls Reference'!A3:A1000)</f>
         <v/>
       </c>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>TABLE 3: CRITICAL FINDINGS REQUIRING IMMEDIATE ATTENTION</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n"/>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="28" t="n"/>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="28" t="n"/>
-      <c r="G16" s="28" t="n"/>
+      <c r="B16" s="21" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="21" t="n"/>
+      <c r="G16" s="21" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Finding</t>
         </is>
       </c>
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Action Required</t>
         </is>
       </c>
-      <c r="D17" s="28" t="n"/>
-      <c r="E17" s="28" t="n"/>
-      <c r="F17" s="28" t="n"/>
-      <c r="G17" s="28" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="21" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="39" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Requirements in gap analysis (no adequate control)</t>
         </is>
       </c>
-      <c r="B18" s="40">
-        <f>COUNTA('Gap Summary'!A3:A1000)</f>
+      <c r="B18" s="33">
+        <f>COUNTA('Gap Summary'!A4:A1000)</f>
         <v/>
       </c>
-      <c r="C18" s="39" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>Review Gap Summary sheet — implement controls or accept risk for each gap item</t>
         </is>
       </c>
-      <c r="D18" s="28" t="n"/>
-      <c r="E18" s="28" t="n"/>
-      <c r="F18" s="28" t="n"/>
-      <c r="G18" s="28" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="21" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="39" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Total requirements not yet mapped</t>
         </is>
       </c>
-      <c r="B19" s="40">
+      <c r="B19" s="33">
         <f>COUNTA('Control Mapping Matrix'!A3:A1000)-COUNTA('Mapping Guidelines'!A3:A1000)</f>
         <v/>
       </c>
-      <c r="C19" s="39" t="inlineStr">
+      <c r="C19" s="32" t="inlineStr">
         <is>
           <t>Complete control mapping for all extracted requirements before gap analysis</t>
         </is>
       </c>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="28" t="n"/>
-      <c r="F19" s="28" t="n"/>
-      <c r="G19" s="28" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="41" t="n"/>
-      <c r="B20" s="41" t="n"/>
-      <c r="C20" s="41" t="n"/>
-      <c r="D20" s="41" t="n"/>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
+      <c r="A20" s="34" t="n"/>
+      <c r="B20" s="34" t="n"/>
+      <c r="C20" s="34" t="n"/>
+      <c r="D20" s="34" t="n"/>
+      <c r="E20" s="34" t="n"/>
+      <c r="F20" s="34" t="n"/>
+      <c r="G20" s="34" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="n"/>
-      <c r="B21" s="41" t="n"/>
-      <c r="C21" s="41" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
-      <c r="G21" s="41" t="n"/>
+      <c r="A21" s="34" t="n"/>
+      <c r="B21" s="34" t="n"/>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="34" t="n"/>
+      <c r="E21" s="34" t="n"/>
+      <c r="F21" s="34" t="n"/>
+      <c r="G21" s="34" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -6837,25 +6704,25 @@
           <t>FINAL DECISION:</t>
         </is>
       </c>
-      <c r="B23" s="41" t="n"/>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="28" t="n"/>
-      <c r="F23" s="28" t="n"/>
-      <c r="G23" s="28" t="n"/>
+      <c r="B23" s="34" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="42" t="inlineStr">
+      <c r="A26" s="35" t="inlineStr">
         <is>
           <t>NEXT REVIEW DETAILS</t>
         </is>
       </c>
-      <c r="B26" s="28" t="n"/>
-      <c r="C26" s="28" t="n"/>
-      <c r="D26" s="28" t="n"/>
-      <c r="E26" s="28" t="n"/>
-      <c r="F26" s="28" t="n"/>
-      <c r="G26" s="28" t="n"/>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="21" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -6863,12 +6730,12 @@
           <t>Next Review Date:</t>
         </is>
       </c>
-      <c r="B27" s="41" t="n"/>
-      <c r="C27" s="28" t="n"/>
-      <c r="D27" s="28" t="n"/>
-      <c r="E27" s="28" t="n"/>
-      <c r="F27" s="28" t="n"/>
-      <c r="G27" s="28" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="21" t="n"/>
+      <c r="G27" s="21" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -6876,12 +6743,12 @@
           <t>Review Responsible:</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n"/>
-      <c r="C28" s="28" t="n"/>
-      <c r="D28" s="28" t="n"/>
-      <c r="E28" s="28" t="n"/>
-      <c r="F28" s="28" t="n"/>
-      <c r="G28" s="28" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -6889,12 +6756,12 @@
           <t>Special Considerations:</t>
         </is>
       </c>
-      <c r="B29" s="41" t="n"/>
-      <c r="C29" s="28" t="n"/>
-      <c r="D29" s="28" t="n"/>
-      <c r="E29" s="28" t="n"/>
-      <c r="F29" s="28" t="n"/>
-      <c r="G29" s="28" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="21" t="n"/>
+      <c r="F29" s="21" t="n"/>
+      <c r="G29" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -6938,7 +6805,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>ASSESSMENT APPROVAL AND SIGN-OFF</t>
         </is>
@@ -6949,7 +6816,7 @@
       <c r="E1" s="6" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="44" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 - Control A.5.31: Legal, Statutory, Regulatory and Contractual Requirements</t>
         </is>
@@ -6960,7 +6827,7 @@
       <c r="E2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="45" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>ASSESSMENT SUMMARY</t>
         </is>
@@ -6991,7 +6858,7 @@
           <t>Assessment Period:</t>
         </is>
       </c>
-      <c r="B5" s="46" t="inlineStr"/>
+      <c r="B5" s="39" t="inlineStr"/>
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
@@ -7002,7 +6869,7 @@
           <t>Overall Compliance Rating:</t>
         </is>
       </c>
-      <c r="B6" s="47">
+      <c r="B6" s="40">
         <f>IFERROR(AVERAGE('Summary Dashboard'!G6:G6),"")</f>
         <v/>
       </c>
@@ -7016,7 +6883,7 @@
           <t>Assessment Status:</t>
         </is>
       </c>
-      <c r="B7" s="46" t="inlineStr"/>
+      <c r="B7" s="39" t="inlineStr"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
@@ -7027,13 +6894,13 @@
           <t>Assessed By:</t>
         </is>
       </c>
-      <c r="B8" s="46" t="inlineStr"/>
+      <c r="B8" s="39" t="inlineStr"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="45" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>COMPLETED BY (ASSESSOR)</t>
         </is>
@@ -7049,7 +6916,7 @@
           <t>Name:</t>
         </is>
       </c>
-      <c r="B12" s="46" t="n"/>
+      <c r="B12" s="39" t="n"/>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
@@ -7060,7 +6927,7 @@
           <t>Title:</t>
         </is>
       </c>
-      <c r="B13" s="46" t="n"/>
+      <c r="B13" s="39" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
@@ -7071,7 +6938,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B14" s="46" t="n"/>
+      <c r="B14" s="39" t="n"/>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
@@ -7082,7 +6949,7 @@
           <t>Signature:</t>
         </is>
       </c>
-      <c r="B15" s="46" t="n"/>
+      <c r="B15" s="39" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
@@ -7093,13 +6960,13 @@
           <t>Comments:</t>
         </is>
       </c>
-      <c r="B16" s="46" t="n"/>
+      <c r="B16" s="39" t="n"/>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="45" t="inlineStr">
+      <c r="A18" s="38" t="inlineStr">
         <is>
           <t>REVIEWED BY (INFORMATION SECURITY OFFICER)</t>
         </is>
@@ -7115,7 +6982,7 @@
           <t>Name:</t>
         </is>
       </c>
-      <c r="B19" s="46" t="n"/>
+      <c r="B19" s="39" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
@@ -7126,7 +6993,7 @@
           <t>Title:</t>
         </is>
       </c>
-      <c r="B20" s="46" t="n"/>
+      <c r="B20" s="39" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
@@ -7137,7 +7004,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B21" s="46" t="n"/>
+      <c r="B21" s="39" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
@@ -7148,7 +7015,7 @@
           <t>Signature:</t>
         </is>
       </c>
-      <c r="B22" s="46" t="n"/>
+      <c r="B22" s="39" t="n"/>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
@@ -7159,13 +7026,13 @@
           <t>Comments:</t>
         </is>
       </c>
-      <c r="B23" s="46" t="n"/>
+      <c r="B23" s="39" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="48" t="inlineStr">
+      <c r="A25" s="41" t="inlineStr">
         <is>
           <t>APPROVED BY (CISO)</t>
         </is>
@@ -7181,7 +7048,7 @@
           <t>Name:</t>
         </is>
       </c>
-      <c r="B26" s="46" t="n"/>
+      <c r="B26" s="39" t="n"/>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
@@ -7192,7 +7059,7 @@
           <t>Title:</t>
         </is>
       </c>
-      <c r="B27" s="46" t="n"/>
+      <c r="B27" s="39" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
@@ -7203,7 +7070,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B28" s="46" t="n"/>
+      <c r="B28" s="39" t="n"/>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="n"/>
@@ -7214,7 +7081,7 @@
           <t>Signature:</t>
         </is>
       </c>
-      <c r="B29" s="46" t="n"/>
+      <c r="B29" s="39" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
@@ -7225,7 +7092,7 @@
           <t>Comments:</t>
         </is>
       </c>
-      <c r="B30" s="46" t="n"/>
+      <c r="B30" s="39" t="n"/>
       <c r="C30" s="6" t="n"/>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
@@ -7236,13 +7103,13 @@
           <t>FINAL DECISION:</t>
         </is>
       </c>
-      <c r="B32" s="46" t="n"/>
+      <c r="B32" s="39" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="6" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="45" t="inlineStr">
+      <c r="A35" s="38" t="inlineStr">
         <is>
           <t>NEXT REVIEW DETAILS</t>
         </is>
@@ -7258,7 +7125,7 @@
           <t>Next Review Date:</t>
         </is>
       </c>
-      <c r="B36" s="46" t="n"/>
+      <c r="B36" s="39" t="n"/>
       <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="6" t="n"/>
@@ -7269,7 +7136,7 @@
           <t>Review Responsible:</t>
         </is>
       </c>
-      <c r="B37" s="46" t="n"/>
+      <c r="B37" s="39" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
@@ -7280,7 +7147,7 @@
           <t>Special Considerations:</t>
         </is>
       </c>
-      <c r="B38" s="46" t="n"/>
+      <c r="B38" s="39" t="n"/>
       <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="n"/>

</xml_diff>